<commit_message>
salvo para não perder o histórico
#### salvo para não perder as análises feitas, mas a partir de agora teremos informações baseadas na cesta de ações e atividades regionalizadas
</commit_message>
<xml_diff>
--- a/R Markdown/resultados/df_anexo_2025.xlsx
+++ b/R Markdown/resultados/df_anexo_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cloudprodamazhotmail-my.sharepoint.com/personal/gabrielmachado_prefeitura_sp_gov_br/Documents/Área de Trabalho/IDRGP/IDRGP-2025/R Markdown/resultados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_27AE5CDE8F79A8D366075C52F37BD272EAD28C58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAB1CCFE-998C-426A-B633-72CE17B0ECB3}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_27AE5CDE8F79A8D366075C52F37BD272EAD28C58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0D415DD-1D10-45C6-844F-D4497E0BB22C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1358,7 +1358,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="58.7109375" customWidth="1"/>
-    <col min="2" max="2" width="56.42578125" customWidth="1"/>
+    <col min="2" max="2" width="80.42578125" customWidth="1"/>
     <col min="3" max="3" width="81.7109375" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>